<commit_message>
index formatting + link prep
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F8731A-F043-5548-A407-33201165CD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CB05E7-F716-D94A-9D5E-97FF0C9D4E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="26800" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="10900" windowWidth="26800" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="30">
   <si>
     <t>week</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t>Mod 11: Survey Sampling</t>
+  </si>
+  <si>
+    <t>1-prep/1.1-prep.qmd</t>
   </si>
 </sst>
 </file>
@@ -524,6 +527,9 @@
       <c r="D2" s="8" t="s">
         <v>16</v>
       </c>
+      <c r="E2" s="7" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1">

</xml_diff>

<commit_message>
fix up 1.2 prep and index
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CB05E7-F716-D94A-9D5E-97FF0C9D4E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13940E2D-E759-EE4D-B3E5-5B98E9ECDF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="10900" windowWidth="26800" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="31">
   <si>
     <t>week</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>1-prep/1.1-prep.qmd</t>
+  </si>
+  <si>
+    <t>1-prep/1.2-prep.qmd</t>
   </si>
 </sst>
 </file>
@@ -545,6 +548,9 @@
       <c r="D3" s="8" t="s">
         <v>16</v>
       </c>
+      <c r="E3" s="7" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1">

</xml_diff>

<commit_message>
activity 1 set *I think*
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942A0768-222F-6343-8113-8C0F3745C36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D804B136-D75D-B04B-86E4-BE536ED31DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="35">
   <si>
     <t>week</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>1-prep/01.2-prep.qmd</t>
+  </si>
+  <si>
+    <t>3-activities/instructions/01.1-activity-turkey-in-pens.qmd</t>
   </si>
 </sst>
 </file>
@@ -548,6 +551,9 @@
       <c r="F2" s="7" t="s">
         <v>30</v>
       </c>
+      <c r="H2" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1">

</xml_diff>

<commit_message>
intro survey + slides
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D804B136-D75D-B04B-86E4-BE536ED31DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DEB8A50-9FE2-A049-A6A0-ADDF9FCC27E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="36">
   <si>
     <t>week</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>3-activities/instructions/01.1-activity-turkey-in-pens.qmd</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1huFMgeDgVDLGn2SQCMUyEFC3V7_B0oH9zRA3VXeGsgk/edit?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -551,6 +554,9 @@
       <c r="F2" s="7" t="s">
         <v>30</v>
       </c>
+      <c r="G2" t="s">
+        <v>35</v>
+      </c>
       <c r="H2" s="7" t="s">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
fix index link and 2.1 prep
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EC4C3A-56F5-3145-A012-DD893FE880FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD24B65A-3E77-1840-ADD3-ED0C51FBFF42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="41">
   <si>
     <t>week</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>2-slides/02.1-crd-design-analysis-model.qmd</t>
+  </si>
+  <si>
+    <t>1-prep/02.1-prep.qmd</t>
   </si>
 </sst>
 </file>
@@ -618,7 +621,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
adding activity 2.2 and fixing some other things up
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9B7577-F227-974E-BD01-0EB8EBC4B728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04FF93EC-3A64-6E4F-9179-816731A7F390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="46">
   <si>
     <t>week</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>2-slides/02.2-crd-contrasts.qmd</t>
+  </si>
+  <si>
+    <t>3-activities/instructions/02.2-activity-comparing-means.qmd</t>
   </si>
 </sst>
 </file>
@@ -665,6 +668,9 @@
       <c r="F5" s="7" t="s">
         <v>44</v>
       </c>
+      <c r="H5" s="7" t="s">
+        <v>45</v>
+      </c>
       <c r="I5" s="7"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
link to class slides
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04FF93EC-3A64-6E4F-9179-816731A7F390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCA9628-625C-1142-B2D1-B273A8CA5B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="47">
   <si>
     <t>week</t>
   </si>
@@ -171,6 +171,9 @@
   </si>
   <si>
     <t>3-activities/instructions/02.2-activity-comparing-means.qmd</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1Ek6Zr9Vd8tYFCtOpWvfTYQTOjVFxCXzuQgJyph8KDSE/edit?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -668,6 +671,9 @@
       <c r="F5" s="7" t="s">
         <v>44</v>
       </c>
+      <c r="G5" t="s">
+        <v>46</v>
+      </c>
       <c r="H5" s="7" t="s">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
midterm 1 practice problems
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E1E834-AD77-EF49-A8C3-A968C721B9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58F1A6C-AF7A-F248-9522-52E54B4958BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="56">
   <si>
     <t>week</t>
   </si>
@@ -198,6 +198,9 @@
   </si>
   <si>
     <t>3-activities/instructions/04.1-activity-contrasts-for-factorials.qmd</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/12ID6VbCZhW5Nx4u54auJqxmrAmgb7ZwLVz-DfXAOtcE/edit?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -753,7 +756,9 @@
       <c r="F7" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G7" s="7"/>
+      <c r="G7" s="7" t="s">
+        <v>55</v>
+      </c>
       <c r="H7" s="7" t="s">
         <v>54</v>
       </c>

</xml_diff>

<commit_message>
3.1 solutions and fixes
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58F1A6C-AF7A-F248-9522-52E54B4958BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A20FA6D-7810-A947-93C3-BBFD31C62842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="57">
   <si>
     <t>week</t>
   </si>
@@ -201,6 +201,9 @@
   </si>
   <si>
     <t>https://docs.google.com/presentation/d/12ID6VbCZhW5Nx4u54auJqxmrAmgb7ZwLVz-DfXAOtcE/edit?usp=sharing</t>
+  </si>
+  <si>
+    <t>6-exams/practice/midterm1-practice.qmd</t>
   </si>
 </sst>
 </file>
@@ -797,7 +800,9 @@
       <c r="D9" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="7"/>
+      <c r="E9" s="7" t="s">
+        <v>56</v>
+      </c>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="I9" s="7"/>

</xml_diff>